<commit_message>
Address QA review: no-JS fallback, a11y, tokens, OG image, meta, fixed XLSX dates, footer links
</commit_message>
<xml_diff>
--- a/public/downloads/coi-tracking-spreadsheet.xlsx
+++ b/public/downloads/coi-tracking-spreadsheet.xlsx
@@ -700,13 +700,13 @@
         <v>1000000</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>46505</v>
+        <v>46954</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>46455</v>
+        <v>46904</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>46605</v>
+        <v>47054</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="N2" s="5" t="n">
-        <v>46705</v>
+        <v>47154</v>
       </c>
       <c r="O2">
         <f>IF(COUNT(G2:I2,N2)=0,"",IF(MIN(G2:I2,N2)&lt;TODAY(),"Expired",IF(MIN(G2:I2,N2)&lt;=TODAY()+30,"Expiring in 30 days","OK")))</f>
@@ -766,10 +766,10 @@
         <v>2000000</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>46325</v>
+        <v>46043</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>46395</v>
+        <v>46113</v>
       </c>
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="3" t="inlineStr">
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="N3" s="5" t="n">
-        <v>46670</v>
+        <v>46388</v>
       </c>
       <c r="O3">
         <f>IF(COUNT(G3:I3,N3)=0,"",IF(MIN(G3:I3,N3)&lt;TODAY(),"Expired",IF(MIN(G3:I3,N3)&lt;=TODAY()+30,"Expiring in 30 days","OK")))</f>
@@ -830,13 +830,13 @@
         <v>1000000</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>46295</v>
+        <v>46013</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>46365</v>
+        <v>46083</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>46365</v>
+        <v>46083</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>

</xml_diff>